<commit_message>
Cambios finales recomendaciones reunion hoy (Sabana a Reporte , Quitar olvide contraseña , admin eximido de timeout y edicion de correo)
</commit_message>
<xml_diff>
--- a/src/main/resources/SABANA_CERTIFICADO_MINI.xlsx
+++ b/src/main/resources/SABANA_CERTIFICADO_MINI.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Proyecto Integrador\certificados-tributarios\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Proyecto Integrador\certificados-tributarios-master\certificados-tributarios\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32855D07-1149-49EA-A344-BBA28774AC0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84AC7F8D-8FE7-4761-AF16-18C6A637580A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{4D3B91EF-504D-40B9-A464-F85D83C5368B}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{4D3B91EF-504D-40B9-A464-F85D83C5368B}"/>
   </bookViews>
   <sheets>
     <sheet name="General (2)" sheetId="3" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="68">
   <si>
     <t>PRIMER_APELLIDO</t>
   </si>
@@ -219,13 +219,37 @@
   </si>
   <si>
     <t>zrinco@hotmail.com</t>
+  </si>
+  <si>
+    <t>coordinacionctic.bga@upb.edu.co</t>
+  </si>
+  <si>
+    <t>jose.serrano.2021@upb.edu.co</t>
+  </si>
+  <si>
+    <t>PEÑA</t>
+  </si>
+  <si>
+    <t>FUENTES</t>
+  </si>
+  <si>
+    <t>JAIRO</t>
+  </si>
+  <si>
+    <t>JOSE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SERRANO </t>
+  </si>
+  <si>
+    <t>PRADA</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -245,6 +269,14 @@
       <color theme="1"/>
       <name val="Calibri Light"/>
       <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -270,10 +302,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -282,8 +315,10 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -596,7 +631,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9F006413-D9B6-48BF-A7B1-A180E4CD51A8}">
-  <dimension ref="A1:S11"/>
+  <dimension ref="A1:S13"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16.6640625" customWidth="1"/>
@@ -604,7 +639,7 @@
     <col min="3" max="3" width="15.88671875" customWidth="1"/>
     <col min="4" max="4" width="27.77734375" customWidth="1"/>
     <col min="5" max="5" width="19.5546875" customWidth="1"/>
-    <col min="6" max="6" width="22.21875" customWidth="1"/>
+    <col min="6" max="6" width="29.109375" customWidth="1"/>
     <col min="7" max="7" width="13.44140625" customWidth="1"/>
     <col min="8" max="8" width="12.44140625" customWidth="1"/>
     <col min="9" max="9" width="12" customWidth="1"/>
@@ -791,7 +826,7 @@
         <v>0</v>
       </c>
       <c r="R3" s="4">
-        <f t="shared" ref="R3:R11" si="0">SUM(G3:Q3)</f>
+        <f t="shared" ref="R3:R12" si="0">SUM(G3:Q3)</f>
         <v>217107</v>
       </c>
       <c r="S3" s="3">
@@ -1278,22 +1313,135 @@
         <v>0</v>
       </c>
     </row>
+    <row r="12" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A12" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E12">
+        <v>1000000001</v>
+      </c>
+      <c r="F12" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="G12" s="3">
+        <v>0</v>
+      </c>
+      <c r="H12" s="3">
+        <v>0</v>
+      </c>
+      <c r="I12" s="3">
+        <v>0</v>
+      </c>
+      <c r="J12" s="3">
+        <v>0</v>
+      </c>
+      <c r="K12" s="3">
+        <v>0</v>
+      </c>
+      <c r="L12" s="3">
+        <v>0</v>
+      </c>
+      <c r="M12" s="3">
+        <v>0</v>
+      </c>
+      <c r="N12" s="3">
+        <v>0</v>
+      </c>
+      <c r="O12" s="3">
+        <v>0</v>
+      </c>
+      <c r="P12" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q12" s="3">
+        <v>0</v>
+      </c>
+      <c r="R12" s="4">
+        <v>0</v>
+      </c>
+      <c r="S12" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A13" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E13">
+        <v>1000000002</v>
+      </c>
+      <c r="F13" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="G13" s="3">
+        <v>0</v>
+      </c>
+      <c r="H13" s="3">
+        <v>0</v>
+      </c>
+      <c r="I13" s="3">
+        <v>0</v>
+      </c>
+      <c r="J13" s="3">
+        <v>0</v>
+      </c>
+      <c r="K13" s="3">
+        <v>0</v>
+      </c>
+      <c r="L13" s="3">
+        <v>0</v>
+      </c>
+      <c r="M13" s="3">
+        <v>0</v>
+      </c>
+      <c r="N13" s="3">
+        <v>0</v>
+      </c>
+      <c r="O13" s="3">
+        <v>0</v>
+      </c>
+      <c r="P13" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q13" s="3">
+        <v>0</v>
+      </c>
+      <c r="R13" s="3">
+        <v>0</v>
+      </c>
+      <c r="S13" s="3">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:S182" xr:uid="{9F006413-D9B6-48BF-A7B1-A180E4CD51A8}"/>
+  <hyperlinks>
+    <hyperlink ref="F12" r:id="rId1" xr:uid="{2957F0C4-3BD4-411C-933E-21B36CD42215}"/>
+    <hyperlink ref="F13" r:id="rId2" xr:uid="{88C929CD-BAD4-47FF-B655-E1A7B3542A6D}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="3b53d3ac-3f50-43a3-baab-349149f6658e">
@@ -1301,6 +1449,15 @@
     </lcf76f155ced4ddcb4097134ff3c332f>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1482,19 +1639,19 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{920BC647-C618-4A23-BBA5-0393A1D7F565}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B03128A5-60ED-4E24-9BBC-8605CD0BF491}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="3b53d3ac-3f50-43a3-baab-349149f6658e"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B03128A5-60ED-4E24-9BBC-8605CD0BF491}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{920BC647-C618-4A23-BBA5-0393A1D7F565}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="3b53d3ac-3f50-43a3-baab-349149f6658e"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>